<commit_message>
v2.26: pensasäänet, pelaajan askeleet −20 % ja ±5 %, terveyspalkkien näkyvyys
- Pensaan läpi heti puska- ja pusikkoääni (2 s tauko), Aarnimetsässä satunnaisesti oksa tai puska; olennoille kahina pensaassa.
- Uudet pelaajan äänet askeleet/puska ja askeleet/oksa (aloitusäänet olentojen kansiosta).
- Pelaajan askeleet 20 % hiljempaa, kaikkien pelaajan äänten voimakkuus vaihtelee ±5 %.
- Terveyspalkki vain suoraan katsottaessa; vahingoittunut myös 10 % ympärillä; vahingon jälkeen 5 s,
  mutta ei jos olento on tosi kaukana ja maaston tai esteiden takana.
- Äänityökalu ei kaadu uuteen ääneen (profiilit + varaprofiili, KORJAUKSET 51), sydämen syke silmukaksi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcnuEGNchuSfRaKmKSwn2M
</commit_message>
<xml_diff>
--- a/sounds/AANILISTA_PELAAJA.xlsx
+++ b/sounds/AANILISTA_PELAAJA.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Osa 3 – pelaajan äänet" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Osa 1 – liike'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Osa 1 – liike'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Osa 2 – toiminnot'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Osa 3 – pelaajan äänet'!$A$1:$G$19</definedName>
   </definedNames>
@@ -470,12 +470,12 @@
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">💧 Vesi</t>
+          <t xml:space="preserve">👣 Askeleet</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">askel_kahlaus</t>
+          <t xml:space="preserve">puska</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="2">
@@ -485,17 +485,17 @@
       </c>
       <c r="E11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">askel_kahlaus_1 (+4 pätkää)</t>
+          <t xml:space="preserve">puska_1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kahlaa matalassa vedessä (joka askeleella)</t>
+          <t xml:space="preserve">kävelet pensaan läpi (heti, enintään 2 s välein) ja satunnaisesti Aarnimetsässä</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">wading water footsteps</t>
+          <t xml:space="preserve">walking through bush rustle, leaves brushing</t>
         </is>
       </c>
     </row>
@@ -507,32 +507,32 @@
       </c>
       <c r="B12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">💧 Vesi</t>
+          <t xml:space="preserve">👣 Askeleet</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">askel_uinti</t>
+          <t xml:space="preserve">oksa</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">✅ valmis (3)</t>
+          <t xml:space="preserve">✅ valmis (2)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">askel_uinti_1, askel_uinti_2, askel_uinti_3</t>
+          <t xml:space="preserve">oksa_1, oksa_2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">uintiveto (noin kerran sekunnissa uidessa)</t>
+          <t xml:space="preserve">oksa rasahtaa satunnaisesti Aarnimetsässä (enintään 2 s välein)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">swimming stroke splash</t>
+          <t xml:space="preserve">twig snap, branch crack footstep</t>
         </is>
       </c>
     </row>
@@ -549,32 +549,106 @@
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">askel_kahlaus</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">✅ valmis (1)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">askel_kahlaus_1 (+4 pätkää)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">kahlaa matalassa vedessä (joka askeleella)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">wading water footsteps</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">💧 Vesi</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">askel_uinti</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">✅ valmis (3)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">askel_uinti_1, askel_uinti_2, askel_uinti_3</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">uintiveto (noin kerran sekunnissa uidessa)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">swimming stroke splash</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">💧 Vesi</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">loiskahdus</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="2">
+      <c r="D15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">✅ valmis (2)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr" s="2">
+      <c r="E15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">loiskahdus_1, loiskahdus_2</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr" s="2">
+      <c r="F15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">menee tai putoaa veteen (kova pudotus = isompi)</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr" s="2">
+      <c r="G15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">splash into water, jump into water</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:G15"/>
 </worksheet>
 </file>
 

</xml_diff>